<commit_message>
pulled mastercode and pushed updated Register
</commit_message>
<xml_diff>
--- a/src/test/resources/DS_ExcelData.xlsx
+++ b/src/test/resources/DS_ExcelData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saphi\eclipse-workspace\DSAlgo_TestNG\src\test\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rresh\eclipse-workspace\DSAlgo_TestNG\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC12C243-B5E5-48DD-86B6-9C36B86B5758}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7D38E27-4F0D-4875-AADB-805B9D0900DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5745" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{B73CB05F-107B-41ED-85A9-C212C46F3310}"/>
+    <workbookView xWindow="1013" yWindow="2242" windowWidth="14400" windowHeight="7373" xr2:uid="{B73CB05F-107B-41ED-85A9-C212C46F3310}"/>
   </bookViews>
   <sheets>
     <sheet name="RegisterPage_Validdata" sheetId="4" r:id="rId1"/>
@@ -183,10 +183,10 @@
 search(arr, 12) </t>
   </si>
   <si>
-    <t>Validrun05</t>
-  </si>
-  <si>
     <t>Invalid user</t>
+  </si>
+  <si>
+    <t>Validruntest03</t>
   </si>
 </sst>
 </file>
@@ -740,7 +740,7 @@
         <v>33</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>21</v>
@@ -864,7 +864,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>11</v>

</xml_diff>